<commit_message>
Actualizar equivalencias: Actualizacion de equivalencias
</commit_message>
<xml_diff>
--- a/equivalencias.xlsx
+++ b/equivalencias.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\libroelec\Equivalencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3C3E82-686F-4DDC-8339-9D3DF4780026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB35193-FFFE-4173-8081-34B87D984C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{299C50DE-1EB3-435D-B7D8-E57BE0EDFFB3}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{299C50DE-1EB3-435D-B7D8-E57BE0EDFFB3}"/>
   </bookViews>
   <sheets>
     <sheet name="afp" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="133">
   <si>
     <t>NO ESTA EN AFP</t>
   </si>
@@ -437,6 +437,15 @@
   </si>
   <si>
     <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
   </si>
 </sst>
 </file>
@@ -533,7 +542,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -566,7 +575,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -937,14 +957,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5890B19D-31C1-476F-B71B-4CC23D1EFB21}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -955,7 +975,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>100</v>
       </c>
@@ -966,7 +986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>6</v>
       </c>
@@ -977,7 +997,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>11</v>
       </c>
@@ -988,7 +1008,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>13</v>
       </c>
@@ -999,7 +1019,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>14</v>
       </c>
@@ -1010,7 +1030,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>19</v>
       </c>
@@ -1021,7 +1041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>31</v>
       </c>
@@ -1032,7 +1052,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>103</v>
       </c>
@@ -1053,14 +1073,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EBF06E0-914A-4224-93AD-1D22B0773178}">
-  <dimension ref="A1:D297"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D321"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.81640625" style="13"/>
-    <col min="3" max="3" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.85546875" style="13"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
         <v>76</v>
       </c>
@@ -1074,7 +1094,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>75</v>
       </c>
@@ -1086,7 +1106,7 @@
       </c>
       <c r="D2" s="10"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>75</v>
       </c>
@@ -1098,7 +1118,7 @@
       </c>
       <c r="D3" s="10"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
@@ -1110,7 +1130,7 @@
       </c>
       <c r="D4" s="10"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>75</v>
       </c>
@@ -1122,7 +1142,7 @@
       </c>
       <c r="D5" s="10"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>75</v>
       </c>
@@ -1134,7 +1154,7 @@
       </c>
       <c r="D6" s="10"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>75</v>
       </c>
@@ -1146,7 +1166,7 @@
       </c>
       <c r="D7" s="10"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>75</v>
       </c>
@@ -1158,7 +1178,7 @@
       </c>
       <c r="D8" s="10"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>75</v>
       </c>
@@ -1170,7 +1190,7 @@
       </c>
       <c r="D9" s="10"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>74</v>
       </c>
@@ -1182,7 +1202,7 @@
       </c>
       <c r="D10" s="10"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>74</v>
       </c>
@@ -1194,7 +1214,7 @@
       </c>
       <c r="D11" s="10"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>74</v>
       </c>
@@ -1206,7 +1226,7 @@
       </c>
       <c r="D12" s="10"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>74</v>
       </c>
@@ -1218,7 +1238,7 @@
       </c>
       <c r="D13" s="10"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>74</v>
       </c>
@@ -1230,7 +1250,7 @@
       </c>
       <c r="D14" s="10"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>74</v>
       </c>
@@ -1242,7 +1262,7 @@
       </c>
       <c r="D15" s="10"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>74</v>
       </c>
@@ -1254,7 +1274,7 @@
       </c>
       <c r="D16" s="10"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>74</v>
       </c>
@@ -1266,7 +1286,7 @@
       </c>
       <c r="D17" s="10"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>73</v>
       </c>
@@ -1278,7 +1298,7 @@
       </c>
       <c r="D18" s="10"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>73</v>
       </c>
@@ -1290,7 +1310,7 @@
       </c>
       <c r="D19" s="10"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>73</v>
       </c>
@@ -1302,7 +1322,7 @@
       </c>
       <c r="D20" s="10"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>73</v>
       </c>
@@ -1314,7 +1334,7 @@
       </c>
       <c r="D21" s="10"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>73</v>
       </c>
@@ -1326,7 +1346,7 @@
       </c>
       <c r="D22" s="10"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>73</v>
       </c>
@@ -1338,7 +1358,7 @@
       </c>
       <c r="D23" s="10"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>73</v>
       </c>
@@ -1350,7 +1370,7 @@
       </c>
       <c r="D24" s="10"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>73</v>
       </c>
@@ -1362,7 +1382,7 @@
       </c>
       <c r="D25" s="10"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>72</v>
       </c>
@@ -1374,7 +1394,7 @@
       </c>
       <c r="D26" s="10"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>72</v>
       </c>
@@ -1386,7 +1406,7 @@
       </c>
       <c r="D27" s="10"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>72</v>
       </c>
@@ -1398,7 +1418,7 @@
       </c>
       <c r="D28" s="10"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>72</v>
       </c>
@@ -1410,7 +1430,7 @@
       </c>
       <c r="D29" s="10"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>72</v>
       </c>
@@ -1422,7 +1442,7 @@
       </c>
       <c r="D30" s="10"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>72</v>
       </c>
@@ -1434,7 +1454,7 @@
       </c>
       <c r="D31" s="10"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>72</v>
       </c>
@@ -1446,7 +1466,7 @@
       </c>
       <c r="D32" s="10"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
         <v>72</v>
       </c>
@@ -1458,7 +1478,7 @@
       </c>
       <c r="D33" s="10"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>71</v>
       </c>
@@ -1470,7 +1490,7 @@
       </c>
       <c r="D34" s="10"/>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
         <v>71</v>
       </c>
@@ -1482,7 +1502,7 @@
       </c>
       <c r="D35" s="10"/>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
         <v>71</v>
       </c>
@@ -1494,7 +1514,7 @@
       </c>
       <c r="D36" s="10"/>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
         <v>71</v>
       </c>
@@ -1506,7 +1526,7 @@
       </c>
       <c r="D37" s="10"/>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>71</v>
       </c>
@@ -1518,7 +1538,7 @@
       </c>
       <c r="D38" s="10"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
         <v>71</v>
       </c>
@@ -1530,7 +1550,7 @@
       </c>
       <c r="D39" s="10"/>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>71</v>
       </c>
@@ -1542,7 +1562,7 @@
       </c>
       <c r="D40" s="10"/>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
         <v>71</v>
       </c>
@@ -1554,7 +1574,7 @@
       </c>
       <c r="D41" s="10"/>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
         <v>70</v>
       </c>
@@ -1566,7 +1586,7 @@
       </c>
       <c r="D42" s="10"/>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
         <v>70</v>
       </c>
@@ -1578,7 +1598,7 @@
       </c>
       <c r="D43" s="10"/>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
         <v>70</v>
       </c>
@@ -1590,7 +1610,7 @@
       </c>
       <c r="D44" s="10"/>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
         <v>70</v>
       </c>
@@ -1602,7 +1622,7 @@
       </c>
       <c r="D45" s="10"/>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>70</v>
       </c>
@@ -1614,7 +1634,7 @@
       </c>
       <c r="D46" s="10"/>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>70</v>
       </c>
@@ -1626,7 +1646,7 @@
       </c>
       <c r="D47" s="10"/>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>70</v>
       </c>
@@ -1638,7 +1658,7 @@
       </c>
       <c r="D48" s="10"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>70</v>
       </c>
@@ -1650,7 +1670,7 @@
       </c>
       <c r="D49" s="10"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>69</v>
       </c>
@@ -1662,7 +1682,7 @@
       </c>
       <c r="D50" s="10"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>69</v>
       </c>
@@ -1674,7 +1694,7 @@
       </c>
       <c r="D51" s="10"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>69</v>
       </c>
@@ -1686,7 +1706,7 @@
       </c>
       <c r="D52" s="10"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>69</v>
       </c>
@@ -1698,7 +1718,7 @@
       </c>
       <c r="D53" s="10"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
         <v>69</v>
       </c>
@@ -1710,7 +1730,7 @@
       </c>
       <c r="D54" s="10"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>69</v>
       </c>
@@ -1722,7 +1742,7 @@
       </c>
       <c r="D55" s="10"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
         <v>69</v>
       </c>
@@ -1734,7 +1754,7 @@
       </c>
       <c r="D56" s="10"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
         <v>69</v>
       </c>
@@ -1746,7 +1766,7 @@
       </c>
       <c r="D57" s="10"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
         <v>68</v>
       </c>
@@ -1758,7 +1778,7 @@
       </c>
       <c r="D58" s="10"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>68</v>
       </c>
@@ -1770,7 +1790,7 @@
       </c>
       <c r="D59" s="10"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>68</v>
       </c>
@@ -1782,7 +1802,7 @@
       </c>
       <c r="D60" s="10"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>68</v>
       </c>
@@ -1794,7 +1814,7 @@
       </c>
       <c r="D61" s="10"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
         <v>68</v>
       </c>
@@ -1806,7 +1826,7 @@
       </c>
       <c r="D62" s="10"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
         <v>68</v>
       </c>
@@ -1818,7 +1838,7 @@
       </c>
       <c r="D63" s="10"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>68</v>
       </c>
@@ -1830,7 +1850,7 @@
       </c>
       <c r="D64" s="10"/>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
         <v>68</v>
       </c>
@@ -1842,7 +1862,7 @@
       </c>
       <c r="D65" s="10"/>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
         <v>67</v>
       </c>
@@ -1854,7 +1874,7 @@
       </c>
       <c r="D66" s="10"/>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>67</v>
       </c>
@@ -1866,7 +1886,7 @@
       </c>
       <c r="D67" s="10"/>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
         <v>67</v>
       </c>
@@ -1878,7 +1898,7 @@
       </c>
       <c r="D68" s="10"/>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
         <v>67</v>
       </c>
@@ -1890,7 +1910,7 @@
       </c>
       <c r="D69" s="10"/>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
         <v>67</v>
       </c>
@@ -1902,7 +1922,7 @@
       </c>
       <c r="D70" s="10"/>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
         <v>67</v>
       </c>
@@ -1914,7 +1934,7 @@
       </c>
       <c r="D71" s="10"/>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
         <v>67</v>
       </c>
@@ -1926,7 +1946,7 @@
       </c>
       <c r="D72" s="10"/>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="s">
         <v>67</v>
       </c>
@@ -1938,7 +1958,7 @@
       </c>
       <c r="D73" s="10"/>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="s">
         <v>66</v>
       </c>
@@ -1950,7 +1970,7 @@
       </c>
       <c r="D74" s="10"/>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="s">
         <v>66</v>
       </c>
@@ -1962,7 +1982,7 @@
       </c>
       <c r="D75" s="10"/>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="s">
         <v>66</v>
       </c>
@@ -1974,7 +1994,7 @@
       </c>
       <c r="D76" s="10"/>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" s="9" t="s">
         <v>66</v>
       </c>
@@ -1986,7 +2006,7 @@
       </c>
       <c r="D77" s="10"/>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
         <v>66</v>
       </c>
@@ -1998,7 +2018,7 @@
       </c>
       <c r="D78" s="10"/>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="s">
         <v>66</v>
       </c>
@@ -2010,7 +2030,7 @@
       </c>
       <c r="D79" s="10"/>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
         <v>66</v>
       </c>
@@ -2022,7 +2042,7 @@
       </c>
       <c r="D80" s="10"/>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" s="9" t="s">
         <v>66</v>
       </c>
@@ -2034,7 +2054,7 @@
       </c>
       <c r="D81" s="10"/>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" s="9" t="s">
         <v>65</v>
       </c>
@@ -2046,7 +2066,7 @@
       </c>
       <c r="D82" s="10"/>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="s">
         <v>65</v>
       </c>
@@ -2058,7 +2078,7 @@
       </c>
       <c r="D83" s="10"/>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="s">
         <v>65</v>
       </c>
@@ -2070,7 +2090,7 @@
       </c>
       <c r="D84" s="10"/>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" s="9" t="s">
         <v>65</v>
       </c>
@@ -2082,7 +2102,7 @@
       </c>
       <c r="D85" s="10"/>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" s="9" t="s">
         <v>65</v>
       </c>
@@ -2094,7 +2114,7 @@
       </c>
       <c r="D86" s="10"/>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="s">
         <v>65</v>
       </c>
@@ -2106,7 +2126,7 @@
       </c>
       <c r="D87" s="10"/>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" s="9" t="s">
         <v>65</v>
       </c>
@@ -2118,7 +2138,7 @@
       </c>
       <c r="D88" s="10"/>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" s="9" t="s">
         <v>65</v>
       </c>
@@ -2130,7 +2150,7 @@
       </c>
       <c r="D89" s="10"/>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" s="9" t="s">
         <v>64</v>
       </c>
@@ -2142,7 +2162,7 @@
       </c>
       <c r="D90" s="10"/>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" s="9" t="s">
         <v>64</v>
       </c>
@@ -2154,7 +2174,7 @@
       </c>
       <c r="D91" s="10"/>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" s="9" t="s">
         <v>64</v>
       </c>
@@ -2166,7 +2186,7 @@
       </c>
       <c r="D92" s="10"/>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" s="9" t="s">
         <v>64</v>
       </c>
@@ -2178,7 +2198,7 @@
       </c>
       <c r="D93" s="10"/>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" s="9" t="s">
         <v>64</v>
       </c>
@@ -2190,7 +2210,7 @@
       </c>
       <c r="D94" s="10"/>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" s="9" t="s">
         <v>64</v>
       </c>
@@ -2202,7 +2222,7 @@
       </c>
       <c r="D95" s="10"/>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="9" t="s">
         <v>64</v>
       </c>
@@ -2214,7 +2234,7 @@
       </c>
       <c r="D96" s="10"/>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="9" t="s">
         <v>64</v>
       </c>
@@ -2226,7 +2246,7 @@
       </c>
       <c r="D97" s="10"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" s="9" t="s">
         <v>63</v>
       </c>
@@ -2238,7 +2258,7 @@
       </c>
       <c r="D98" s="10"/>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="9" t="s">
         <v>63</v>
       </c>
@@ -2250,7 +2270,7 @@
       </c>
       <c r="D99" s="10"/>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" s="9" t="s">
         <v>63</v>
       </c>
@@ -2262,7 +2282,7 @@
       </c>
       <c r="D100" s="10"/>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="9" t="s">
         <v>63</v>
       </c>
@@ -2274,7 +2294,7 @@
       </c>
       <c r="D101" s="10"/>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" s="9" t="s">
         <v>63</v>
       </c>
@@ -2286,7 +2306,7 @@
       </c>
       <c r="D102" s="10"/>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" s="9" t="s">
         <v>63</v>
       </c>
@@ -2298,7 +2318,7 @@
       </c>
       <c r="D103" s="10"/>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="9" t="s">
         <v>63</v>
       </c>
@@ -2310,7 +2330,7 @@
       </c>
       <c r="D104" s="10"/>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A105" s="9" t="s">
         <v>63</v>
       </c>
@@ -2322,7 +2342,7 @@
       </c>
       <c r="D105" s="10"/>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" s="9" t="s">
         <v>62</v>
       </c>
@@ -2334,7 +2354,7 @@
       </c>
       <c r="D106" s="10"/>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A107" s="9" t="s">
         <v>62</v>
       </c>
@@ -2346,7 +2366,7 @@
       </c>
       <c r="D107" s="10"/>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" s="9" t="s">
         <v>62</v>
       </c>
@@ -2358,7 +2378,7 @@
       </c>
       <c r="D108" s="10"/>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A109" s="9" t="s">
         <v>62</v>
       </c>
@@ -2370,7 +2390,7 @@
       </c>
       <c r="D109" s="10"/>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A110" s="9" t="s">
         <v>62</v>
       </c>
@@ -2382,7 +2402,7 @@
       </c>
       <c r="D110" s="10"/>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A111" s="9" t="s">
         <v>62</v>
       </c>
@@ -2394,7 +2414,7 @@
       </c>
       <c r="D111" s="10"/>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A112" s="9" t="s">
         <v>62</v>
       </c>
@@ -2406,7 +2426,7 @@
       </c>
       <c r="D112" s="10"/>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A113" s="9" t="s">
         <v>62</v>
       </c>
@@ -2418,7 +2438,7 @@
       </c>
       <c r="D113" s="10"/>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A114" s="9" t="s">
         <v>61</v>
       </c>
@@ -2430,7 +2450,7 @@
       </c>
       <c r="D114" s="10"/>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A115" s="9" t="s">
         <v>61</v>
       </c>
@@ -2442,7 +2462,7 @@
       </c>
       <c r="D115" s="10"/>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A116" s="9" t="s">
         <v>61</v>
       </c>
@@ -2454,7 +2474,7 @@
       </c>
       <c r="D116" s="10"/>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="9" t="s">
         <v>61</v>
       </c>
@@ -2466,7 +2486,7 @@
       </c>
       <c r="D117" s="10"/>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="9" t="s">
         <v>61</v>
       </c>
@@ -2478,7 +2498,7 @@
       </c>
       <c r="D118" s="10"/>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A119" s="9" t="s">
         <v>61</v>
       </c>
@@ -2490,7 +2510,7 @@
       </c>
       <c r="D119" s="10"/>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A120" s="9" t="s">
         <v>61</v>
       </c>
@@ -2502,7 +2522,7 @@
       </c>
       <c r="D120" s="10"/>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A121" s="9" t="s">
         <v>61</v>
       </c>
@@ -2514,7 +2534,7 @@
       </c>
       <c r="D121" s="10"/>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A122" s="9" t="s">
         <v>60</v>
       </c>
@@ -2526,7 +2546,7 @@
       </c>
       <c r="D122" s="10"/>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A123" s="9" t="s">
         <v>60</v>
       </c>
@@ -2538,7 +2558,7 @@
       </c>
       <c r="D123" s="10"/>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A124" s="9" t="s">
         <v>60</v>
       </c>
@@ -2550,7 +2570,7 @@
       </c>
       <c r="D124" s="10"/>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A125" s="9" t="s">
         <v>60</v>
       </c>
@@ -2562,7 +2582,7 @@
       </c>
       <c r="D125" s="10"/>
     </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A126" s="9" t="s">
         <v>60</v>
       </c>
@@ -2574,7 +2594,7 @@
       </c>
       <c r="D126" s="10"/>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A127" s="9" t="s">
         <v>60</v>
       </c>
@@ -2586,7 +2606,7 @@
       </c>
       <c r="D127" s="10"/>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A128" s="9" t="s">
         <v>60</v>
       </c>
@@ -2598,7 +2618,7 @@
       </c>
       <c r="D128" s="10"/>
     </row>
-    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A129" s="9" t="s">
         <v>60</v>
       </c>
@@ -2610,7 +2630,7 @@
       </c>
       <c r="D129" s="10"/>
     </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A130" s="9" t="s">
         <v>59</v>
       </c>
@@ -2622,7 +2642,7 @@
       </c>
       <c r="D130" s="10"/>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A131" s="9" t="s">
         <v>59</v>
       </c>
@@ -2634,7 +2654,7 @@
       </c>
       <c r="D131" s="10"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A132" s="9" t="s">
         <v>59</v>
       </c>
@@ -2646,7 +2666,7 @@
       </c>
       <c r="D132" s="10"/>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A133" s="9" t="s">
         <v>59</v>
       </c>
@@ -2658,7 +2678,7 @@
       </c>
       <c r="D133" s="10"/>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A134" s="9" t="s">
         <v>59</v>
       </c>
@@ -2670,7 +2690,7 @@
       </c>
       <c r="D134" s="10"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A135" s="9" t="s">
         <v>59</v>
       </c>
@@ -2682,7 +2702,7 @@
       </c>
       <c r="D135" s="10"/>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="9" t="s">
         <v>59</v>
       </c>
@@ -2694,7 +2714,7 @@
       </c>
       <c r="D136" s="10"/>
     </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="9" t="s">
         <v>59</v>
       </c>
@@ -2706,7 +2726,7 @@
       </c>
       <c r="D137" s="10"/>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A138" s="9" t="s">
         <v>58</v>
       </c>
@@ -2718,7 +2738,7 @@
       </c>
       <c r="D138" s="10"/>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A139" s="9" t="s">
         <v>58</v>
       </c>
@@ -2730,7 +2750,7 @@
       </c>
       <c r="D139" s="10"/>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A140" s="9" t="s">
         <v>58</v>
       </c>
@@ -2742,7 +2762,7 @@
       </c>
       <c r="D140" s="10"/>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A141" s="9" t="s">
         <v>58</v>
       </c>
@@ -2754,7 +2774,7 @@
       </c>
       <c r="D141" s="10"/>
     </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="9" t="s">
         <v>58</v>
       </c>
@@ -2766,7 +2786,7 @@
       </c>
       <c r="D142" s="10"/>
     </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="9" t="s">
         <v>58</v>
       </c>
@@ -2778,7 +2798,7 @@
       </c>
       <c r="D143" s="10"/>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A144" s="9" t="s">
         <v>58</v>
       </c>
@@ -2790,7 +2810,7 @@
       </c>
       <c r="D144" s="10"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A145" s="9" t="s">
         <v>58</v>
       </c>
@@ -2802,7 +2822,7 @@
       </c>
       <c r="D145" s="10"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A146" s="9" t="s">
         <v>57</v>
       </c>
@@ -2814,7 +2834,7 @@
       </c>
       <c r="D146" s="10"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="9" t="s">
         <v>57</v>
       </c>
@@ -2826,7 +2846,7 @@
       </c>
       <c r="D147" s="10"/>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A148" s="9" t="s">
         <v>57</v>
       </c>
@@ -2838,7 +2858,7 @@
       </c>
       <c r="D148" s="10"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A149" s="9" t="s">
         <v>57</v>
       </c>
@@ -2850,7 +2870,7 @@
       </c>
       <c r="D149" s="10"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A150" s="9" t="s">
         <v>57</v>
       </c>
@@ -2862,7 +2882,7 @@
       </c>
       <c r="D150" s="10"/>
     </row>
-    <row r="151" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A151" s="9" t="s">
         <v>57</v>
       </c>
@@ -2874,7 +2894,7 @@
       </c>
       <c r="D151" s="10"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A152" s="9" t="s">
         <v>57</v>
       </c>
@@ -2886,7 +2906,7 @@
       </c>
       <c r="D152" s="10"/>
     </row>
-    <row r="153" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A153" s="9" t="s">
         <v>57</v>
       </c>
@@ -2898,7 +2918,7 @@
       </c>
       <c r="D153" s="10"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A154" s="9" t="s">
         <v>56</v>
       </c>
@@ -2910,7 +2930,7 @@
       </c>
       <c r="D154" s="10"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A155" s="9" t="s">
         <v>56</v>
       </c>
@@ -2922,7 +2942,7 @@
       </c>
       <c r="D155" s="10"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A156" s="9" t="s">
         <v>56</v>
       </c>
@@ -2934,7 +2954,7 @@
       </c>
       <c r="D156" s="10"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A157" s="9" t="s">
         <v>56</v>
       </c>
@@ -2946,7 +2966,7 @@
       </c>
       <c r="D157" s="10"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A158" s="9" t="s">
         <v>56</v>
       </c>
@@ -2958,7 +2978,7 @@
       </c>
       <c r="D158" s="10"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A159" s="9" t="s">
         <v>56</v>
       </c>
@@ -2970,7 +2990,7 @@
       </c>
       <c r="D159" s="10"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A160" s="9" t="s">
         <v>56</v>
       </c>
@@ -2982,7 +3002,7 @@
       </c>
       <c r="D160" s="10"/>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="9" t="s">
         <v>56</v>
       </c>
@@ -2994,7 +3014,7 @@
       </c>
       <c r="D161" s="10"/>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="9" t="s">
         <v>55</v>
       </c>
@@ -3006,7 +3026,7 @@
       </c>
       <c r="D162" s="10"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A163" s="9" t="s">
         <v>55</v>
       </c>
@@ -3018,7 +3038,7 @@
       </c>
       <c r="D163" s="10"/>
     </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A164" s="9" t="s">
         <v>55</v>
       </c>
@@ -3030,7 +3050,7 @@
       </c>
       <c r="D164" s="10"/>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A165" s="9" t="s">
         <v>55</v>
       </c>
@@ -3042,7 +3062,7 @@
       </c>
       <c r="D165" s="10"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A166" s="9" t="s">
         <v>55</v>
       </c>
@@ -3054,7 +3074,7 @@
       </c>
       <c r="D166" s="10"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A167" s="9" t="s">
         <v>55</v>
       </c>
@@ -3066,7 +3086,7 @@
       </c>
       <c r="D167" s="10"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A168" s="9" t="s">
         <v>55</v>
       </c>
@@ -3078,7 +3098,7 @@
       </c>
       <c r="D168" s="10"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A169" s="9" t="s">
         <v>55</v>
       </c>
@@ -3090,7 +3110,7 @@
       </c>
       <c r="D169" s="10"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A170" s="9" t="s">
         <v>54</v>
       </c>
@@ -3100,7 +3120,7 @@
       <c r="C170" s="2"/>
       <c r="D170" s="10"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A171" s="9" t="s">
         <v>54</v>
       </c>
@@ -3112,7 +3132,7 @@
       </c>
       <c r="D171" s="10"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A172" s="9" t="s">
         <v>54</v>
       </c>
@@ -3124,7 +3144,7 @@
       </c>
       <c r="D172" s="10"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A173" s="9" t="s">
         <v>54</v>
       </c>
@@ -3136,7 +3156,7 @@
       </c>
       <c r="D173" s="10"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A174" s="9" t="s">
         <v>54</v>
       </c>
@@ -3148,7 +3168,7 @@
       </c>
       <c r="D174" s="10"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A175" s="9" t="s">
         <v>54</v>
       </c>
@@ -3160,7 +3180,7 @@
       </c>
       <c r="D175" s="10"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A176" s="9" t="s">
         <v>54</v>
       </c>
@@ -3172,7 +3192,7 @@
       </c>
       <c r="D176" s="10"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A177" s="9" t="s">
         <v>54</v>
       </c>
@@ -3184,7 +3204,7 @@
       </c>
       <c r="D177" s="10"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A178" s="9" t="s">
         <v>53</v>
       </c>
@@ -3196,7 +3216,7 @@
       </c>
       <c r="D178" s="10"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A179" s="9" t="s">
         <v>53</v>
       </c>
@@ -3208,7 +3228,7 @@
       </c>
       <c r="D179" s="10"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A180" s="9" t="s">
         <v>53</v>
       </c>
@@ -3220,7 +3240,7 @@
       </c>
       <c r="D180" s="10"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A181" s="9" t="s">
         <v>53</v>
       </c>
@@ -3232,7 +3252,7 @@
       </c>
       <c r="D181" s="10"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A182" s="9" t="s">
         <v>53</v>
       </c>
@@ -3244,7 +3264,7 @@
       </c>
       <c r="D182" s="10"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A183" s="9" t="s">
         <v>53</v>
       </c>
@@ -3256,7 +3276,7 @@
       </c>
       <c r="D183" s="10"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="9" t="s">
         <v>53</v>
       </c>
@@ -3268,7 +3288,7 @@
       </c>
       <c r="D184" s="10"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A185" s="9" t="s">
         <v>53</v>
       </c>
@@ -3280,7 +3300,7 @@
       </c>
       <c r="D185" s="10"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A186" s="9" t="s">
         <v>52</v>
       </c>
@@ -3292,7 +3312,7 @@
       </c>
       <c r="D186" s="10"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A187" s="9" t="s">
         <v>52</v>
       </c>
@@ -3304,7 +3324,7 @@
       </c>
       <c r="D187" s="10"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A188" s="9" t="s">
         <v>52</v>
       </c>
@@ -3316,7 +3336,7 @@
       </c>
       <c r="D188" s="10"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A189" s="9" t="s">
         <v>52</v>
       </c>
@@ -3328,7 +3348,7 @@
       </c>
       <c r="D189" s="10"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A190" s="9" t="s">
         <v>52</v>
       </c>
@@ -3340,7 +3360,7 @@
       </c>
       <c r="D190" s="10"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A191" s="9" t="s">
         <v>52</v>
       </c>
@@ -3352,7 +3372,7 @@
       </c>
       <c r="D191" s="10"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="9" t="s">
         <v>52</v>
       </c>
@@ -3364,7 +3384,7 @@
       </c>
       <c r="D192" s="10"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A193" s="9" t="s">
         <v>52</v>
       </c>
@@ -3376,7 +3396,7 @@
       </c>
       <c r="D193" s="10"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A194" s="9" t="s">
         <v>51</v>
       </c>
@@ -3390,7 +3410,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A195" s="9" t="s">
         <v>51</v>
       </c>
@@ -3404,7 +3424,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A196" s="9" t="s">
         <v>51</v>
       </c>
@@ -3418,7 +3438,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A197" s="9" t="s">
         <v>51</v>
       </c>
@@ -3432,7 +3452,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A198" s="9" t="s">
         <v>51</v>
       </c>
@@ -3446,7 +3466,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A199" s="9" t="s">
         <v>51</v>
       </c>
@@ -3460,7 +3480,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A200" s="9" t="s">
         <v>51</v>
       </c>
@@ -3474,7 +3494,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A201" s="9" t="s">
         <v>51</v>
       </c>
@@ -3488,7 +3508,7 @@
         <v>5059065</v>
       </c>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="9" t="s">
         <v>50</v>
       </c>
@@ -3502,7 +3522,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A203" s="9" t="s">
         <v>50</v>
       </c>
@@ -3516,7 +3536,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A204" s="9" t="s">
         <v>50</v>
       </c>
@@ -3530,7 +3550,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A205" s="9" t="s">
         <v>50</v>
       </c>
@@ -3544,7 +3564,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A206" s="9" t="s">
         <v>50</v>
       </c>
@@ -3558,7 +3578,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A207" s="9" t="s">
         <v>50</v>
       </c>
@@ -3572,7 +3592,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A208" s="9" t="s">
         <v>50</v>
       </c>
@@ -3586,7 +3606,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A209" s="9" t="s">
         <v>50</v>
       </c>
@@ -3600,7 +3620,7 @@
         <v>5097663</v>
       </c>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A210" s="9" t="s">
         <v>49</v>
       </c>
@@ -3614,7 +3634,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A211" s="9" t="s">
         <v>49</v>
       </c>
@@ -3628,7 +3648,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A212" s="9" t="s">
         <v>49</v>
       </c>
@@ -3642,7 +3662,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="9" t="s">
         <v>49</v>
       </c>
@@ -3656,7 +3676,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A214" s="9" t="s">
         <v>49</v>
       </c>
@@ -3670,7 +3690,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A215" s="9" t="s">
         <v>49</v>
       </c>
@@ -3684,7 +3704,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="9" t="s">
         <v>49</v>
       </c>
@@ -3698,7 +3718,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="9" t="s">
         <v>49</v>
       </c>
@@ -3712,7 +3732,7 @@
         <v>5130133</v>
       </c>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="14" t="s">
         <v>118</v>
       </c>
@@ -3726,7 +3746,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="219" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A219" s="14" t="s">
         <v>118</v>
       </c>
@@ -3740,7 +3760,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="220" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A220" s="14" t="s">
         <v>118</v>
       </c>
@@ -3754,7 +3774,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="221" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A221" s="14" t="s">
         <v>118</v>
       </c>
@@ -3768,7 +3788,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="222" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="14" t="s">
         <v>118</v>
       </c>
@@ -3782,7 +3802,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="223" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A223" s="14" t="s">
         <v>118</v>
       </c>
@@ -3796,7 +3816,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="224" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A224" s="14" t="s">
         <v>118</v>
       </c>
@@ -3810,7 +3830,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="225" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A225" s="14" t="s">
         <v>118</v>
       </c>
@@ -3824,7 +3844,7 @@
         <v>5154047</v>
       </c>
     </row>
-    <row r="226" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A226" s="14" t="s">
         <v>120</v>
       </c>
@@ -3838,7 +3858,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="227" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A227" s="14" t="s">
         <v>120</v>
       </c>
@@ -3852,7 +3872,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="228" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A228" s="14" t="s">
         <v>120</v>
       </c>
@@ -3866,7 +3886,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="229" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A229" s="14" t="s">
         <v>120</v>
       </c>
@@ -3880,7 +3900,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="230" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A230" s="14" t="s">
         <v>120</v>
       </c>
@@ -3894,7 +3914,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="231" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A231" s="14" t="s">
         <v>120</v>
       </c>
@@ -3908,7 +3928,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="232" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A232" s="14" t="s">
         <v>120</v>
       </c>
@@ -3922,7 +3942,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="233" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A233" s="14" t="s">
         <v>120</v>
       </c>
@@ -3936,7 +3956,7 @@
         <v>5169088</v>
       </c>
     </row>
-    <row r="234" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A234" s="14" t="s">
         <v>121</v>
       </c>
@@ -3950,7 +3970,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="235" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" s="14" t="s">
         <v>121</v>
       </c>
@@ -3964,7 +3984,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="236" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" s="14" t="s">
         <v>121</v>
       </c>
@@ -3978,7 +3998,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="237" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A237" s="14" t="s">
         <v>121</v>
       </c>
@@ -3992,7 +4012,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="238" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A238" s="14" t="s">
         <v>121</v>
       </c>
@@ -4006,7 +4026,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="239" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A239" s="14" t="s">
         <v>121</v>
       </c>
@@ -4020,7 +4040,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="240" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A240" s="14" t="s">
         <v>121</v>
       </c>
@@ -4034,7 +4054,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="241" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A241" s="14" t="s">
         <v>121</v>
       </c>
@@ -4048,7 +4068,7 @@
         <v>5179327</v>
       </c>
     </row>
-    <row r="242" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A242" s="14" t="s">
         <v>123</v>
       </c>
@@ -4062,7 +4082,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="243" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A243" s="14" t="s">
         <v>123</v>
       </c>
@@ -4076,7 +4096,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="244" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A244" s="14" t="s">
         <v>123</v>
       </c>
@@ -4090,7 +4110,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="245" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A245" s="14" t="s">
         <v>123</v>
       </c>
@@ -4104,7 +4124,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="246" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" s="14" t="s">
         <v>123</v>
       </c>
@@ -4118,7 +4138,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="247" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A247" s="14" t="s">
         <v>123</v>
       </c>
@@ -4132,7 +4152,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="248" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A248" s="14" t="s">
         <v>123</v>
       </c>
@@ -4146,7 +4166,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="249" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A249" s="14" t="s">
         <v>123</v>
       </c>
@@ -4160,7 +4180,7 @@
         <v>5167711</v>
       </c>
     </row>
-    <row r="250" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" s="14" t="s">
         <v>124</v>
       </c>
@@ -4174,7 +4194,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="251" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A251" s="14" t="s">
         <v>124</v>
       </c>
@@ -4188,7 +4208,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="252" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A252" s="14" t="s">
         <v>124</v>
       </c>
@@ -4202,7 +4222,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="253" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A253" s="14" t="s">
         <v>124</v>
       </c>
@@ -4216,7 +4236,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="254" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" s="14" t="s">
         <v>124</v>
       </c>
@@ -4230,7 +4250,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="255" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A255" s="14" t="s">
         <v>124</v>
       </c>
@@ -4244,7 +4264,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="256" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A256" s="14" t="s">
         <v>124</v>
       </c>
@@ -4258,7 +4278,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="257" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" s="14" t="s">
         <v>124</v>
       </c>
@@ -4272,7 +4292,7 @@
         <v>5194627</v>
       </c>
     </row>
-    <row r="258" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" s="14" t="s">
         <v>125</v>
       </c>
@@ -4286,7 +4306,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="259" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" s="14" t="s">
         <v>125</v>
       </c>
@@ -4300,7 +4320,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="260" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" s="14" t="s">
         <v>125</v>
       </c>
@@ -4314,7 +4334,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="261" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" s="14" t="s">
         <v>125</v>
       </c>
@@ -4328,7 +4348,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="262" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" s="14" t="s">
         <v>125</v>
       </c>
@@ -4342,7 +4362,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="263" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" s="14" t="s">
         <v>125</v>
       </c>
@@ -4356,7 +4376,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="264" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" s="14" t="s">
         <v>125</v>
       </c>
@@ -4370,7 +4390,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="265" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" s="14" t="s">
         <v>125</v>
       </c>
@@ -4384,7 +4404,7 @@
         <v>5208157</v>
       </c>
     </row>
-    <row r="266" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" s="14" t="s">
         <v>126</v>
       </c>
@@ -4398,7 +4418,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="267" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="14" t="s">
         <v>126</v>
       </c>
@@ -4412,7 +4432,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="268" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" s="14" t="s">
         <v>126</v>
       </c>
@@ -4426,7 +4446,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="269" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" s="14" t="s">
         <v>126</v>
       </c>
@@ -4440,7 +4460,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="270" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" s="14" t="s">
         <v>126</v>
       </c>
@@ -4454,7 +4474,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="271" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" s="14" t="s">
         <v>126</v>
       </c>
@@ -4468,7 +4488,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="272" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" s="14" t="s">
         <v>126</v>
       </c>
@@ -4482,7 +4502,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="273" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" s="14" t="s">
         <v>126</v>
       </c>
@@ -4496,7 +4516,7 @@
         <v>5222933</v>
       </c>
     </row>
-    <row r="274" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" s="14" t="s">
         <v>127</v>
       </c>
@@ -4507,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="D274" s="10">
-        <v>5222933</v>
-      </c>
-    </row>
-    <row r="275" spans="1:4" x14ac:dyDescent="0.35">
+        <v>5228990</v>
+      </c>
+    </row>
+    <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" s="14" t="s">
         <v>127</v>
       </c>
@@ -4524,7 +4544,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="276" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" s="14" t="s">
         <v>127</v>
       </c>
@@ -4538,7 +4558,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="277" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" s="14" t="s">
         <v>127</v>
       </c>
@@ -4552,7 +4572,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="278" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" s="14" t="s">
         <v>127</v>
       </c>
@@ -4566,7 +4586,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="279" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" s="14" t="s">
         <v>127</v>
       </c>
@@ -4580,7 +4600,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="280" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" s="14" t="s">
         <v>127</v>
       </c>
@@ -4594,7 +4614,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="281" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" s="14" t="s">
         <v>127</v>
       </c>
@@ -4608,7 +4628,7 @@
         <v>5228990</v>
       </c>
     </row>
-    <row r="282" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" s="14" t="s">
         <v>128</v>
       </c>
@@ -4622,7 +4642,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="283" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" s="14" t="s">
         <v>128</v>
       </c>
@@ -4636,7 +4656,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="284" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" s="14" t="s">
         <v>128</v>
       </c>
@@ -4650,7 +4670,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="285" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" s="14" t="s">
         <v>128</v>
       </c>
@@ -4664,7 +4684,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="286" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" s="14" t="s">
         <v>128</v>
       </c>
@@ -4678,7 +4698,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="287" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" s="14" t="s">
         <v>128</v>
       </c>
@@ -4692,7 +4712,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="288" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" s="14" t="s">
         <v>128</v>
       </c>
@@ -4706,7 +4726,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="289" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" s="14" t="s">
         <v>128</v>
       </c>
@@ -4720,7 +4740,7 @@
         <v>5240118</v>
       </c>
     </row>
-    <row r="290" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" s="14" t="s">
         <v>129</v>
       </c>
@@ -4731,10 +4751,10 @@
         <v>0</v>
       </c>
       <c r="D290" s="10">
-        <v>5240118</v>
-      </c>
-    </row>
-    <row r="291" spans="1:4" x14ac:dyDescent="0.35">
+        <v>5364290</v>
+      </c>
+    </row>
+    <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" s="14" t="s">
         <v>129</v>
       </c>
@@ -4748,7 +4768,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="292" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" s="14" t="s">
         <v>129</v>
       </c>
@@ -4762,7 +4782,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="293" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" s="14" t="s">
         <v>129</v>
       </c>
@@ -4776,7 +4796,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="294" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" s="14" t="s">
         <v>129</v>
       </c>
@@ -4790,7 +4810,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="295" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" s="14" t="s">
         <v>129</v>
       </c>
@@ -4804,7 +4824,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="296" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" s="14" t="s">
         <v>129</v>
       </c>
@@ -4818,7 +4838,7 @@
         <v>5364290</v>
       </c>
     </row>
-    <row r="297" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" s="14" t="s">
         <v>129</v>
       </c>
@@ -4830,6 +4850,342 @@
       </c>
       <c r="D297" s="10">
         <v>5364290</v>
+      </c>
+    </row>
+    <row r="298" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A298" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B298" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C298" s="15">
+        <v>0</v>
+      </c>
+      <c r="D298" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="299" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A299" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B299" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C299" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D299" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="300" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A300" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B300" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C300" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D300" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="301" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A301" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B301" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C301" s="2">
+        <v>11.27</v>
+      </c>
+      <c r="D301" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="302" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A302" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B302" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C302" s="2">
+        <v>11.16</v>
+      </c>
+      <c r="D302" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="303" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A303" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B303" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C303" s="2">
+        <v>11.45</v>
+      </c>
+      <c r="D303" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="304" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A304" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B304" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C304" s="2">
+        <v>10.58</v>
+      </c>
+      <c r="D304" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="305" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A305" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="B305" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C305" s="2">
+        <v>10.46</v>
+      </c>
+      <c r="D305" s="10">
+        <v>5379593</v>
+      </c>
+    </row>
+    <row r="306" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A306" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B306" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C306" s="15">
+        <v>0</v>
+      </c>
+      <c r="D306" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="307" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A307" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B307" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C307" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D307" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="308" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A308" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B308" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C308" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D308" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="309" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A309" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B309" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C309" s="2">
+        <v>11.27</v>
+      </c>
+      <c r="D309" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="310" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A310" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B310" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C310" s="2">
+        <v>11.16</v>
+      </c>
+      <c r="D310" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="311" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A311" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B311" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C311" s="2">
+        <v>11.45</v>
+      </c>
+      <c r="D311" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="312" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A312" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B312" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C312" s="2">
+        <v>10.58</v>
+      </c>
+      <c r="D312" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="313" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A313" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="B313" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C313" s="2">
+        <v>10.46</v>
+      </c>
+      <c r="D313" s="10">
+        <v>5386601</v>
+      </c>
+    </row>
+    <row r="314" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A314" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B314" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C314" s="15">
+        <v>0</v>
+      </c>
+      <c r="D314" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="315" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A315" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B315" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C315" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D315" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="316" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A316" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B316" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C316" s="2">
+        <v>11.44</v>
+      </c>
+      <c r="D316" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="317" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A317" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B317" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C317" s="2">
+        <v>11.27</v>
+      </c>
+      <c r="D317" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="318" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A318" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B318" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C318" s="2">
+        <v>11.16</v>
+      </c>
+      <c r="D318" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="319" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A319" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B319" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C319" s="2">
+        <v>11.45</v>
+      </c>
+      <c r="D319" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="320" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A320" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B320" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C320" s="2">
+        <v>10.58</v>
+      </c>
+      <c r="D320" s="10">
+        <v>5424251</v>
+      </c>
+    </row>
+    <row r="321" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A321" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="B321" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C321" s="2">
+        <v>10.46</v>
+      </c>
+      <c r="D321" s="10">
+        <v>5424251</v>
       </c>
     </row>
   </sheetData>
@@ -4844,14 +5200,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47F3E9E6-B7F6-412E-B601-0B1132924FD0}">
   <dimension ref="A1:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -4862,7 +5218,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -4873,7 +5229,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>3</v>
       </c>
@@ -4884,7 +5240,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>4</v>
       </c>
@@ -4895,7 +5251,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>9</v>
       </c>
@@ -4906,7 +5262,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>12</v>
       </c>
@@ -4917,7 +5273,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>37</v>
       </c>
@@ -4928,7 +5284,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>38</v>
       </c>
@@ -4939,7 +5295,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>39</v>
       </c>
@@ -4950,7 +5306,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>40</v>
       </c>
@@ -4961,7 +5317,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>41</v>
       </c>
@@ -4970,7 +5326,7 @@
       </c>
       <c r="C11" s="2"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>42</v>
       </c>
@@ -4979,7 +5335,7 @@
       </c>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>43</v>
       </c>
@@ -4990,7 +5346,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>102</v>
       </c>
@@ -5001,7 +5357,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2" t="s">
         <v>40</v>
@@ -5010,7 +5366,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2" t="s">
         <v>42</v>
@@ -5019,7 +5375,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
         <v>44</v>
@@ -5043,13 +5399,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCCD0E17-004C-4DC3-A7EF-BAE0650EA11F}">
-  <dimension ref="A1:B34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B41"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
@@ -5057,7 +5413,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>75</v>
       </c>
@@ -5065,7 +5421,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>74</v>
       </c>
@@ -5073,7 +5429,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>73</v>
       </c>
@@ -5081,7 +5437,7 @@
         <v>1.55</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>72</v>
       </c>
@@ -5089,7 +5445,7 @@
         <v>1.61</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>71</v>
       </c>
@@ -5097,7 +5453,7 @@
         <v>1.61</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>70</v>
       </c>
@@ -5105,7 +5461,7 @@
         <v>1.61</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>69</v>
       </c>
@@ -5113,7 +5469,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>68</v>
       </c>
@@ -5121,7 +5477,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>67</v>
       </c>
@@ -5129,7 +5485,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>66</v>
       </c>
@@ -5137,7 +5493,7 @@
         <v>1.47</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>65</v>
       </c>
@@ -5145,7 +5501,7 @@
         <v>1.47</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>64</v>
       </c>
@@ -5153,7 +5509,7 @@
         <v>1.47</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>63</v>
       </c>
@@ -5161,7 +5517,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>62</v>
       </c>
@@ -5169,7 +5525,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>61</v>
       </c>
@@ -5177,7 +5533,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>60</v>
       </c>
@@ -5185,7 +5541,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>59</v>
       </c>
@@ -5193,7 +5549,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>58</v>
       </c>
@@ -5201,7 +5557,7 @@
         <v>1.49</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>57</v>
       </c>
@@ -5209,7 +5565,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>56</v>
       </c>
@@ -5217,7 +5573,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>55</v>
       </c>
@@ -5225,7 +5581,7 @@
         <v>2.0099999999999998</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>54</v>
       </c>
@@ -5233,7 +5589,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>53</v>
       </c>
@@ -5241,7 +5597,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>52</v>
       </c>
@@ -5249,7 +5605,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>51</v>
       </c>
@@ -5257,7 +5613,7 @@
         <v>1.38</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>50</v>
       </c>
@@ -5265,7 +5621,7 @@
         <v>1.38</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>49</v>
       </c>
@@ -5273,7 +5629,7 @@
         <v>1.38</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>118</v>
       </c>
@@ -5281,7 +5637,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>120</v>
       </c>
@@ -5289,7 +5645,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>121</v>
       </c>
@@ -5297,7 +5653,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>123</v>
       </c>
@@ -5305,7 +5661,7 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>124</v>
       </c>
@@ -5313,12 +5669,68 @@
         <v>1.88</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
         <v>125</v>
       </c>
       <c r="B34" s="3">
         <v>1.88</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B35" s="3">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" s="3">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B37" s="3">
+        <v>1.49</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B38" s="16">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="16">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="16">
+        <v>1.54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="B41" s="10">
+        <v>1.62</v>
       </c>
     </row>
   </sheetData>
@@ -5333,13 +5745,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E681D62B-E25D-4202-85FE-FFC2CD4633F5}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="2.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -5350,7 +5762,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -5361,7 +5773,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -5372,7 +5784,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -5383,7 +5795,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -5402,12 +5814,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5039E4F-6049-4E52-B46B-343C87FDD2E5}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -5418,7 +5830,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6">
         <v>0</v>
       </c>
@@ -5429,7 +5841,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="6">
         <v>1</v>
       </c>
@@ -5440,7 +5852,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="6">
         <v>2</v>
       </c>
@@ -5451,7 +5863,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6">
         <v>3</v>
       </c>
@@ -5462,7 +5874,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>4</v>
       </c>
@@ -5473,7 +5885,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6"/>
       <c r="B7" s="7" t="s">
         <v>96</v>
@@ -5489,10 +5901,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F62DD568-BA2F-495E-8ABF-7EF2EE834C81}">
-  <dimension ref="A1:B26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:B30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>119</v>
       </c>
@@ -5500,7 +5912,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>63</v>
       </c>
@@ -5508,7 +5920,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>62</v>
       </c>
@@ -5516,7 +5928,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>61</v>
       </c>
@@ -5524,7 +5936,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>60</v>
       </c>
@@ -5532,7 +5944,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>59</v>
       </c>
@@ -5540,7 +5952,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>58</v>
       </c>
@@ -5548,7 +5960,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>57</v>
       </c>
@@ -5556,7 +5968,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>56</v>
       </c>
@@ -5564,7 +5976,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>55</v>
       </c>
@@ -5572,133 +5984,161 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="18">
         <v>5.4</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="18">
         <v>5.4</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="18">
         <v>5.4</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="18">
         <v>3.1</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="18">
         <v>5.2</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B24">
+      <c r="B24" s="18">
         <v>4.5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B25">
+      <c r="B25" s="18">
         <v>4.5</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" s="16" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="B26">
+      <c r="B26" s="19">
         <v>3.1</v>
       </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="B27" s="18">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="18">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="20" t="s">
+        <v>132</v>
+      </c>
+      <c r="B29" s="18">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B14">
@@ -5712,14 +6152,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C50F2F9C-A0EF-4427-96D4-C74F9D093DCF}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -5730,7 +6170,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>101</v>
       </c>
@@ -5741,7 +6181,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>201</v>
       </c>
@@ -5752,7 +6192,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>301</v>
       </c>
@@ -5763,7 +6203,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>401</v>
       </c>
@@ -5774,7 +6214,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>402</v>
       </c>
@@ -5785,7 +6225,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>403</v>
       </c>
@@ -5796,7 +6236,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>404</v>
       </c>
@@ -5807,7 +6247,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>405</v>
       </c>
@@ -5818,7 +6258,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>406</v>
       </c>
@@ -5829,7 +6269,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>407</v>
       </c>
@@ -5840,7 +6280,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>408</v>
       </c>
@@ -5851,7 +6291,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>409</v>
       </c>
@@ -5862,7 +6302,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>410</v>
       </c>
@@ -5873,7 +6313,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>411</v>
       </c>
@@ -5884,7 +6324,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>412</v>
       </c>
@@ -5895,7 +6335,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>501</v>
       </c>
@@ -5906,7 +6346,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>601</v>
       </c>
@@ -5917,7 +6357,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>701</v>
       </c>

</xml_diff>